<commit_message>
Name the join-key column, rename all download filenames to site+date
- Template's blank purple join-key column now has a real header,
  "Cell ID + Base Station Name", instead of being blank (which pandas
  read as "Unnamed: 2" in the Previous Reports table view). Located by
  name now in huawei_automation.py instead of fragile column-position
  detection.
- All download buttons (Generate Report's immediate download for both
  ZTE and Huawei, and Previous Reports') now use a clear
  "zte_<date>.xlsx" / "huawei_<date>.xlsx" filename instead of the
  previous inconsistent/ambiguous names (e.g. a bare "2026-08-25.xlsx"
  that didn't say which site type it was).
</commit_message>
<xml_diff>
--- a/template/huawei_configuration.xlsx
+++ b/template/huawei_configuration.xlsx
@@ -28989,7 +28989,11 @@
           <t>Base Station Name</t>
         </is>
       </c>
-      <c r="C1" s="5" t="n"/>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Cell ID + Base Station Name</t>
+        </is>
+      </c>
       <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Cell ID</t>

</xml_diff>